<commit_message>
RF-3309: feedback matrix v2 — verbatim comments, PO scope calls applied
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DpzepkLYwCzujeEtvjJxcF
</commit_message>
<xml_diff>
--- a/docs/brd/RF-3309/RF-3309_HoR_feedback_matrix.xlsx
+++ b/docs/brd/RF-3309/RF-3309_HoR_feedback_matrix.xlsx
@@ -36,7 +36,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -50,7 +50,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F2F7FA"/>
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4E4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -80,7 +95,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -88,13 +103,16 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -465,16 +483,16 @@
   <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="70" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="58" customWidth="1" min="1" max="1"/>
+    <col width="62" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Business requirements (Head of Retail)</t>
+          <t>Business requirements — original comment (Fadel Mansour, verbatim)</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -484,7 +502,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Incorporated in BRD v1.1 (Yes/No)</t>
+          <t>Incorporated in BRD v1.1</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -496,12 +514,16 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>1. Employer selection and validation</t>
+          <t>1. Employer selection and validation
+The Employer Name should not operate as an unrestricted free-text field wherever this can be avoided. The preferred design should allow the Credit user to search and select the employer from the approved Employer Master / Empaneled Company List.
+If free text amendment is required as an exception, the system should require additional validation before the updated employer can affect ALOC, DBR, income multiplier, eligibility or limit.
+Please also define the employer matching logic, including Such as Exact match, Fuzzy match / confidence threshold., Arabic and English employer names, Trade name versus legal name, Employer aliases, Duplicate employer records, Active/inactive employer status.
+The BRD currently states that the updated name will be matched against the Empaneled Company List and the classification rerun. This needs to be more explicitly controlled</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Partially Covered + Development. The matching logic he asks to control is the live platform logic the edit re-uses: the amended name is matched against the Empaneled Company List via the bank's matching tool with a 0.9 confidence threshold, Category &lt;&gt; NON-ALOC, and active-status check — classification is never taken from the typed text itself (BRD section 3, system action 2). Search-and-select from the Empaneled Company List with free text only as a flagged exception is NEW front-end scope — recommended to accept: it raises STP and removes typo risk. Matching-rule documentation (exact/fuzzy threshold, trade vs legal name, aliases, Arabic names, duplicates, active status) to be written out explicitly; alias/Arabic coverage depends on Employer Master data quality (item 10).</t>
+          <t>Accepted — Development. Search-and-select over the Empaneled Company List replaces the free-text field; free text remains only as a flagged exception. The matching logic he asks to control is the live platform logic the edit already re-uses (match against the Empaneled Company List at 0.9 confidence threshold, Category &lt;&gt; NON-ALOC, active status — classification is never taken from the typed text); it will be written out explicitly. Alias / Arabic coverage depends on Employer Master data quality (item 10).</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -511,261 +533,293 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>BRD v1.1: section 2 redesigned — employer picker over the Empaneled Company List + exception free-text path; section 3 adds the explicit matching-rules table. Today's screen: SC3 (single Company Name field) will be replaced. Effort: FE picker + validation = medium.</t>
+          <t>BRD v1.1: section 2 redesigned (employer picker + exception free-text path, SC3 re-rendered); explicit matching-rules table added to section 3. The classification mechanics themselves: no change (BRD v1.0 section 3, system action 2).</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>2. Source validation before applying the amendment</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>Partially Covered + Decision required (Credit/Risk). The design is already validation-first in the classification sense: a manual name cannot by itself create ALOC — ALOC results only from an independent system match against the approved Empaneled list (BRD section 3, action 2; SC5 shows the re-classified result with match %). What is new: validating the amendment against EFR / salary / employment-certificate evidence. System-side EFR re-validation is a new integration (high effort); recommended middle ground — mandatory supporting-evidence reference captured with the amendment (links to item 3/12), manual evidence check by Credit user, no new integration in phase 1. Scope of acceptable evidence to be decided by Credit/Risk.</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>2. Source validation before applying the amendment
+The employer amendment should follow a validation-first model.
+Where available, the amended employer should be validated against the relevant authoritative or supporting source, such as EFR / government employment record, salary information, employment certificate, pays lip or any other approved source used by the Bank.
+A manual amendment by the Credit user should not, by itself, be sufficient to establish a more favorable employer classification.</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Already satisfied in substance — the design is validation-first: a manually typed name can never by itself establish ALOC; the classification results only from the independent system match against the approved Empaneled Company List (BRD v1.0 section 3, action 2; SC5 shows the re-classified result with match score). New: a supporting-evidence reference captured with the amendment; system-side EFR / document validation would be a new integration and is not proposed for this scope.</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>BRD v1.1: validation-first principle stated verbatim (his highlighted text); evidence-reference field added to the edit section; classification independence already shown in section 3 + SC4 note. Decision owner: Credit/Risk on evidence list.</t>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>BRD v1.1: validation-first principle stated verbatim + evidence-reference field. Classification independence: no change (already v1.0).</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>3. Mandatory reason for change</t>
+          <t>3. Mandatory reason for change
+Every Employer Name amendment must require a mandatory reason code.
+Suggested reasons: Spelling correction, Employer legal name / trade name correction, Employer alias, EFR / government record mismatch, Employer Master mapping issue, Customer-provided information correction &amp; Other. (If Other is selected, a mandatory comment should be required)</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Accepted — Development (small). Supersedes the earlier working decision to mirror the existing Edit sections (which carry no reason field). Reason-code dropdown with his suggested values + mandatory comment when Other; reason recorded in the audit trail and available to MIS.</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>PUSH BACK. Consistent platform behaviour: none of the live Credit Queue Edit sections (Finalized Income, Liability Info, Length of Service, Other Income and Expenses) carries a reason field, and the amendment cannot of itself improve the classification (see item 2) — the control value of a reason code is limited while the full old-to-new trail, user and timestamp are already recorded in the Application History (BRD v1.0 section 3 action 6, SC6). A reason code adds friction to every correction without changing any system decision.</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>No — pushed back</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>BRD v1.1: reason code + comment added to the Employment Information section (SC3 to be re-rendered) and to the audit-trail fields (section 3 action 6, SC6).</t>
+          <t>No change to BRD. Fallback if insisted: reason dropdown is small development — can be added in v1.1 without redesign.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>4. STP versus exception handling</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>Accepted — Development (medium). The current flow is exactly his STP leg (matched -&gt; auto re-run -&gt; routing, BRD sections 3 and 6). Controlled STP and Exception legs are new control logic; recommended to map them onto the existing Credit Queue L1/L2/L3 authority levels and queue routing rather than a new workflow: material positive impact -&gt; approval at the applicable delegated-authority level; unmatched/conflicting/repeat cases -&gt; manual-review routing.</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>BRD v1.1: STP decision matrix table added (STP / Controlled STP / Exception with triggering conditions and target queue/authority). Builds on flow diagram + section 6 summary.</t>
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>4. STP versus exception handling
+Please define a clear STP decision matrix.
+The expected design should be:
+STP: Employer successfully matched and validated, no conflicting information and no exception criteria triggered -&gt; automatically update the employer, rerun classification, recalculation, Rule Engine and routing.
+Controlled STP: Employer is validated, but the amendment creates a material positive credit impact -&gt; system performs the recalculation automatically but applies the relevant Credit approval level / delegated authority.
+Exception: Employer cannot be confidently matched, evidence conflicts, repeated amendments are detected, or other risk conditions are triggered -&gt; application should move to manual review rather than allowing an unrestricted override.</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>NOT IN SCOPE of this feature. This feature delivers the capability to edit the Employer Name and re-run the existing logic (classification, recalculation, Rule Engine, routing) — which is exactly the STP leg he describes, already in BRD v1.0 sections 3 and 6. A Controlled-STP / Exception decision matrix with delegated-authority routing is a broader credit-workflow design to be discussed as a new scope, not inside this change. Note the edit already happens inside the manual Credit Queue, operated by authorised Credit users under the existing L1/L2/L3 authority model.</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>No — new scope</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>STP leg: no change (v1.0 flow diagram + sections 3, 6). Decision matrix / authority routing: separate scope discussion.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>5. Material positive credit impact</t>
+          <t>5. Material positive credit impact
+The system must identify whenever the employer amendment creates a more favorable credit position, including where it: Changes N-ALOC to ALOC. Moves the employer into a more favorable category. Increases permitted DBR. Increases income multiplier. Increases approved/proposed limit. Removes a deviation. Converts an otherwise ineligible application into an eligible application.
+These cases should be specifically controlled and visible to the approving Credit user.</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Accepted — Development (medium). All seven impact signals are values the re-run already recalculates (classification, category, DBR, multiplier, limit, deviations, eligibility — BRD section 3 actions 2–4). New scope is detecting the favourable delta and surfacing it to the approving Credit user (before/after comparison), feeding the Controlled-STP leg of item 4.</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>NOT IN SCOPE of this feature — belongs to the same new-scope discussion as item 4. All seven values are already recalculated and displayed to the Credit user after the re-run (ALOC with match score, category, Rule Engine Result, Approve Limit Result — BRD v1.0 sections 3-4, SC5), and the before/after record is in the Application History (SC6). Automated favourable-delta detection with approval gating is new control logic for the new scope.</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>No — new scope</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>BRD v1.1: impact-detection rule + before/after display for the approver; ties to the audit fields of item 12. SC5 (Application Details after update) extended with the comparison view.</t>
+          <t>Visibility of recalculated results: no change (v1.0 SC5/SC6). Impact-detection control: new scope with item 4.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>6. Repeat employer amendments</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>Accepted — Development (small/medium). Supersedes the baseline 'no cap on repeat edits'. Configurable repeat-amendment control: first correction per the standard flow; any subsequent amendment triggers higher authority (queue escalation), fresh reason capture and monitoring visibility (item 9).</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>BRD v1.1: repeat-amendment rule replaces the 'no cap' statement (was in section 3 bullet); every edit already writes its own history step (SC6) so the full trail exists.</t>
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>6. Repeat employer amendments
+The current BRD states that there is no cap on repeat edits.
+Please revise this requirement.
+Unlimited employer amendments are not recommended where the employer classification directly impacts DBR, multiplier and limit assignment.
+The system should have a configurable control over repeat amendments. At minimum, any subsequent amendment after the initial correction should trigger additional authority, reason capture and appropriate monitoring.</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>PUSH BACK. Repeat edits are already bounded and fully visible: every edit re-runs the Rule Engine under the existing shared re-run counter — more than 2 Rule Engine failures auto-rejects the application (BRD v1.0 section 3 action 4) — and every edit writes its own Edit Information step with the full old-to-new trail (SC6). The edit is performed by authorised Credit users inside the controlled queue; additional authority for repeats belongs to the item 4 new-scope discussion if pursued.</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>No — pushed back</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>No change to BRD (v1.0 already documents counter + per-edit audit). Fallback: configurable repeat threshold is feasible if the bank insists.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>7. Rule Engine rerun counter</t>
+          <t>7. Rule Engine rerun counter
+Please ensure that: Technical/integration failures do not consume the business rerun counter. Only genuine business-rule failures are counted where appropriate. The customer is not rejected because of a system timeout, API failure or technical retry.</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Covered with clarification. The shared counter (existing platform behaviour, unchanged by this feature — BRD section 3 action 4) counts business rule-engine failures of the application, not technical errors; technical/integration failures follow the failure-handling path (item 15) and are not business rejections. To be stated explicitly so a timeout can never consume the counter or reject the customer.</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>Agreed — this is already the behaviour: the counter counts business Rule Engine failures of the application (existing platform rule, unchanged by this feature); technical/integration failures follow error handling and never consume the counter or reject the customer. One clarification sentence added so it is explicit.</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>No change</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>BRD v1.1: action 4 reworded — business failures only; technical failure -&gt; retry/recovery per the new resiliency section, counter untouched.</t>
+          <t>BRD v1.0 section 3 action 4 (existing shared counter); v1.1 adds one clarification sentence only.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>8. AML / KYC impact</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>Decision required — Compliance. Current documented treatment (BRD section 5): no re-screening on the edit; the corrected name reaches the screening system through the post-decision CIF-update call. This is consistent with every existing Edit section. Confirmation to be obtained from Compliance and the agreed logic documented; if employer data is part of KYC risk profiling, the refresh trigger will be specified by Compliance.</t>
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>8. AML / KYC impact
+The BRD currently states that AML screening will not be rerun following an employer amendment.
+Please reconfirm this treatment with Compliance and clearly document the agreed logic.
+If employer information forms part of customer risk assessment, KYC profiling or screening, the appropriate refresh/reassessment should be triggered.</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>The treatment is documented in BRD v1.0 section 5: no re-screening on the edit — consistent with every existing Edit section — and the corrected name reaches the screening system through the post-decision CIF-update call. Confirmation to be obtained from Compliance; the documented logic stands unless Compliance directs otherwise.</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>BRD v1.1 keeps the documented logic with an explicit 'treatment confirmed by Compliance on [date]' placeholder. Owner: Compliance. Covered today in section 5 downstream table.</t>
+          <t>No change</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>BRD v1.0 section 5 (EastNets row). Action: Compliance confirmation — owner Compliance; v1.1 adds a 'confirmed by Compliance on [date]' placeholder only.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>9. Fraud monitoring</t>
+          <t>9. Fraud monitoring
+Please include employer amendments in the fraud/control monitoring framework.
+At minimum, the system should make available for monitoring Number of employer amendments per application, Amendments by Credit user, N-ALOC to ALOC changes, Employer-category upgrades, Resulting limit increases, Repeated amendment to the same employers, Unusual concentration of amendments by a particular user.</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Accepted — Development (reporting, small). The enhanced audit trail (item 12) already captures every data point his monitoring list needs (amendments per application/user, N-ALOC-&gt;ALOC changes, category upgrades, limit movement, repeats). Recommended delivery: a monitoring dataset/report extract over the audit data rather than a new framework.</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>PUSH BACK on new framework scope. Every data point listed is already captured per edit in the audit trail / Application History (user, timestamps, old/new name and classification — BRD v1.0 section 3 action 6, SC6) and is extractable for monitoring from day one. A dedicated fraud-monitoring capability / dashboards is reporting scope to be planned with item 18, not part of this change.</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>No — new scope</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>BRD v1.1: monitoring dataset defined from the audit-trail fields; folded into one MIS section with item 18. Source data visible today in SC6 history.</t>
+          <t>Monitoring source data: no change (v1.0 audit trail). Monitoring reports: new scope with item 18.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>10. Employer Master governance</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>Out of this CR — separate change. Ownership, maker-checker and data model (IDs, aliases, Arabic names, effective dates) of the Empaneled Company List are governance of a bank-owned master that exists today with its own upload/maintenance process. Recommended: raise as a separate Employer Master Governance CR; this feature consumes the master as-is and inherits every improvement automatically.</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>Referenced in BRD v1.1 dependencies only. Note: alias/Arabic matching quality (item 1) depends on this stream.</t>
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>10. Employer Master governance
+Please define the ownership and governance of the Employer Master / Empaneled Company List.
+This should cover Employer ID if available, Legal name, Trade name, Arabic/English names, Aliases, ALOC classification, Category, Industry/sector, Effective date and Active/inactive status.
+Maker-checker for employer-master changes.</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Out of this feature — the Empaneled Company List is a bank-owned master that exists today with its own upload and maintenance process; its governance, data model and maker-checker are a separate change request. This feature consumes the master as-is and automatically inherits every improvement made to it.</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>No — separate CR</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Referenced in BRD dependencies only. Alias/Arabic matching quality (item 1) depends on this stream.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>11. Source hierarchy</t>
+          <t>11. Source hierarchy
+The BRD should clearly distinguish between Customer-declared Employer Name, Original system-derived Employer Name, Validated Employer Name and Credit-amended Employer Name.
+The original source should never be lost or overwritten.
+Please also define the source hierarchy so downstream users can clearly understand which employer information has been used for the final credit decision.</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Covered — documentation strengthened. The four values he lists already exist as distinct, never-overwritten data points: customer-declared (Customer Journey input), system-derived original (kept as Original Employer Name at first edit), validated/finalized (the working value), credit-amended (source = Credit Department, Updated By/On) — BRD sections 3 (action 1) and 4; visible in SC5 (Company Name Source row).</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
+          <t>Already covered: the four values exist as distinct, never-overwritten data points — customer-declared (Customer Journey input, never modified), system-derived original (kept at first edit), finalized working value, credit-amended (Source = Credit Department with Updated By/On) — BRD v1.0 section 3 action 1 and section 4; visible in SC5 (Company Name Source row). The finalized value is the single value used for the credit decision (section 5).</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>No change</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>BRD v1.0 sections 3, 4, 5 + SC5. v1.1 adds only a one-glance hierarchy table naming the same values.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>12. Enhanced audit trail
+Please expand it to capture at minimum Old Employer Name, New Employer Name, Old/new Employer ID, Old/new source, Old/new ALOC status/category, Old/new DBR, Old/new income multiplier, Old/new proposed/approved limit, Reason for amendment, Supporting evidence/reference where applicable, User ID/email, Date/time, Rule Engine version and Result of the re-evaluation.</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Accepted — Development (small). Baseline already records old/new name, old source, old/new ALOC, user and timestamps on labelled lines (BRD v1.0 section 3 action 6, SC6). Extension adds employer ID, DBR, multiplier, limit, evidence reference, Rule Engine version and re-evaluation result — all values the re-run already produces. (Reason field follows the item 3 outcome.)</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>BRD v1.1: explicit source-hierarchy table added to section 4 naming which value drives the credit decision (the finalized value) and which are preserved references.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>12. Enhanced audit trail</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>Accepted — Development (small/medium). Baseline already records old/new name, old source, old/new ALOC, user, date/time on separate labelled lines (BRD section 3 action 6; SC6). Extension: old/new employer ID, DBR, income multiplier, proposed/approved limit, reason code, evidence reference, Rule Engine version, re-evaluation result — all values produced by the re-run.</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>BRD v1.1: audit field list expanded in section 3 action 6; SC6 step detail re-rendered with the fuller record.</t>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>BRD v1.1: audit field list expanded; SC6 re-rendered. Base trail: no change (v1.0).</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>13. Atomic processing / rollback</t>
+          <t>13. Atomic processing / rollback
+All employer-related changes must be processed as one atomic transaction.
+The Employer Name should not be successfully updated while the classification, limit assignment or Rule Engine remains on the previous value.
+If any part of the recalculation or integration fails, the system should either Roll back completely to the last successful state; or Hold the application in a controlled pending/error status for recovery. Partial updates should not be permitted.</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Accepted — stated explicitly (his second highlighted requirement, verbatim). Baseline already locks the application during the run (section 3 action 7); v1.1 adds: one controlled transaction across name/classification/variables/limit/RE/routing, no partial commit, rollback to last successful state or controlled recovery status on failure.</t>
+          <t>Accepted — his highlighted transaction paragraph is adopted verbatim. Locking during the run already exists (BRD v1.0 section 3 action 7); v1.1 makes the one-controlled-transaction / no-partial-commit / rollback-or-recovery rule explicit.</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
@@ -775,41 +829,44 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>BRD v1.1: atomic-transaction clause added to section 3; recovery status defined with item 15.</t>
+          <t>BRD v1.1: atomic-transaction clause in section 3; recovery status defined with item 15. Locking: no change (v1.0 action 7).</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>14. Concurrency and locking</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>Covered — strengthened. Locking and the 'Application is in another request processing' behaviour are in section 3 action 7. Added: simultaneous-edit prevention, stale-session protection and version check before save.</t>
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>14. Concurrency and locking
+Please strengthen this further by ensuring that: Two users cannot update the employer simultaneously, A stale screen/session cannot overwrite a more recent employer update and Proper version/concurrency validation exists before saving.</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Already covered in principle: the application is locked during processing and a concurrent action gets 'The Application is in another request processing.' (BRD v1.0 section 3 action 7). v1.1 adds the stale-session / version-check wording.</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>BRD v1.1: action 7 extended with optimistic-concurrency/version validation wording.</t>
+          <t>No change</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>BRD v1.0 section 3 action 7; v1.1 adds one strengthening sentence (version validation before save).</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>15. Failure handling and resiliency</t>
+          <t>15. Failure handling and resiliency
+Please add explicit handling for Employer-classification service failure, Rule Engine timeout, Integration/API timeout, Duplicate submission, Retry, Idempotency, Partial processing and Recovery/reconciliation.
+A technical failure should not leave the application in an inconsistent state.</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Accepted — new NFR section. Explicit handling for classification-service failure, RE timeout, integration timeout, duplicate submission, retry, idempotency, partial processing, recovery/reconciliation; no inconsistent state (pairs with items 7 and 13).</t>
+          <t>Accepted — new non-functional section covering the listed failure modes, idempotency and recovery; pairs with items 7 and 13 (technical failures never consume the business counter; no partial state).</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
@@ -819,95 +876,103 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>BRD v1.1: new 'Failure handling and resiliency' section; effort owned by engineering estimate.</t>
+          <t>BRD v1.1: new 'Failure handling and resiliency' section; engineering to size.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>16. Downstream consistency</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>Covered. Section 5 is exactly this: every consumer (CAM, Affordability Form, document stack, all application views, core banking, screening) reads the single finalized value after the update. The explicit one-sentence requirement he asks for will be added above the table.</t>
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>16. Downstream consistency
+Please add an explicit requirement that all downstream systems and documents must consume the same finalized Employer Name and classification following a successful update.
+There should be no situation where one system shows the original employer while another uses the amended employer for credit decisioning.</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Already covered — this is exactly BRD v1.0 section 5: every consumer (application views across all queues and enquiry, CAM, Affordability Assessment Form, document stack, core banking, screening) reads the single finalized value after the update. The explicit one-sentence requirement is added above the table.</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>BRD v1.1: explicit consistency statement added to section 5; no scope change.</t>
+          <t>No change</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>BRD v1.0 section 5 (downstream consumers table); v1.1 adds the one-sentence explicit requirement only.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>17. Customer-declared information</t>
+          <t>17. Customer-declared information
+I agree with the current approach that the original Application Form should continue to retain what the customer originally submitted.
+However, internally the system should clearly distinguish between: Customer Declared Employer and Bank Validated Employer.
+The customer declaration should never be overwritten.</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Covered — he agrees with the approach. The Application Form remains the customer's OTP-time record (section 5), the Customer Journey input is never modified (section 3 action 1), and the Customer-Declared vs Bank-Validated distinction is carried by the source hierarchy of item 11.</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>Agreed by Head of Retail — already the design: the Application Form stays the customer's OTP-time record and the Customer Journey input is never modified (BRD v1.0 sections 3 and 5); the Customer-Declared vs Bank-Validated distinction is carried by the source data points of item 11.</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>No change</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>BRD v1.1: terminology 'Customer Declared Employer / Bank Validated Employer' adopted in the section 4 hierarchy table.</t>
+          <t>BRD v1.0 sections 3, 5; v1.1 adopts the 'Customer Declared / Bank Validated' terminology in the item 11 table.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>18. MIS and management reporting</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>Accepted — Development (reporting) with phasing decision. Report pack (amendments by user/employer, old/new classification, limit movement, STP %, exception %, repeats, outcomes, reason codes) builds on the same audit dataset as item 9. Recommended: define the dataset in v1.1, deliver reports as a phased MIS item sized with engineering.</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>BRD v1.1: MIS section defining the reporting dataset; delivery phasing to be agreed in planning (one MIS section covers items 9 + 18).</t>
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>18. MIS and management reporting
+Please include appropriate MIS / reporting capability covering Employer amendments by user, Employer amendments by employer, Old/new classification, Limit uplift/downward movement, Percentage processed STP, Percentage routed to exceptions, Repeat amendments, Approval/rejection outcome &amp; Reason codes.</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>PUSH BACK on scope. The reporting dataset is derivable from the enhanced audit trail (item 12) from day one; a dedicated MIS / report pack is reporting scope to be planned separately together with item 9 — not part of this change. STP/exception percentages additionally depend on the item 4 new-scope decision matrix.</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>No — new scope</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Source dataset: covered by items 12 / v1.0 audit trail. Report delivery: separate reporting scope with item 9.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Explicit requirements (highlighted): validation-first exception-based model; one controlled transaction</t>
+          <t>Explicit requirements (highlighted paragraphs)
+Employer Name amendment shall follow a validation-first, exception-based model. Manual amendment shall not by itself establish employer eligibility or classification. The system shall independently validate the amended employer against approved Employer Master data [...] Where validation is successful and no exception criteria are triggered, processing shall continue STP. Where the amendment results in an unverified employer, ambiguous match, material positive credit impact, repeated amendment or conflicting source information, the application shall automatically route to the applicable control/approval queue.
+The Employer Name update, employer classification, calculated variables, limit assignment, Rule Engine execution and routing shall be treated as one controlled transaction. In case of any failure, no partial update shall be committed [...].</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Accepted verbatim. Both highlighted paragraphs are compatible with the approved architecture and will be carried word-for-word as governing requirements — they summarise items 1, 2, 4, 5 and 13.</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>Partially accepted. The validation-first principle and the one-controlled-transaction paragraph are adopted (items 2 and 13 — the first is already how classification works, the second is made explicit). The exception-routing clause (material positive impact / repeated amendment -&gt; control queue) follows the items 4-6 outcome — new scope / pushed back as above.</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>BRD v1.1: both paragraphs added as the governing requirement at the top of the end-to-end section.</t>
+          <t>Validation-first + atomic transaction: in v1.1. Exception-routing clause: follows the item 4 new-scope discussion.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
RF-3309: feedback matrix v3 — PO business-language responses, platform-grounded positions
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DpzepkLYwCzujeEtvjJxcF
</commit_message>
<xml_diff>
--- a/docs/brd/RF-3309/RF-3309_HoR_feedback_matrix.xlsx
+++ b/docs/brd/RF-3309/RF-3309_HoR_feedback_matrix.xlsx
@@ -36,7 +36,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -51,11 +51,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E2EFDA"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FCE4E4"/>
       </patternFill>
     </fill>
     <fill>
@@ -95,7 +90,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -110,9 +105,6 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -483,16 +475,16 @@
   <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="58" customWidth="1" min="1" max="1"/>
-    <col width="62" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="46" customWidth="1" min="4" max="4"/>
+    <col width="56" customWidth="1" min="1" max="1"/>
+    <col width="66" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Business requirements — original comment (Fadel Mansour, verbatim)</t>
+          <t>Business requirements — original comment (verbatim)</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -523,7 +515,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Accepted — Development. Search-and-select over the Empaneled Company List replaces the free-text field; free text remains only as a flagged exception. The matching logic he asks to control is the live platform logic the edit already re-uses (match against the Empaneled Company List at 0.9 confidence threshold, Category &lt;&gt; NON-ALOC, active status — classification is never taken from the typed text); it will be written out explicitly. Alias / Arabic coverage depends on Employer Master data quality (item 10).</t>
+          <t>Agreed. The design will be updated so the Credit user searches and selects the employer from the Empaneled Company List, with free-text entry kept only as an exception path. One point of clarity: the matching and classification logic is not new to this feature — it is the Day-1 platform logic (name matching against the Empaneled Company List at a 90% confidence threshold, company category and active status checks), and the edit simply re-runs it. We will document these matching rules explicitly in the BRD. Coverage of aliases, Arabic names and duplicates is a function of the Empaneled Company List data itself and is addressed under item 10.</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -533,7 +525,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>BRD v1.1: section 2 redesigned (employer picker + exception free-text path, SC3 re-rendered); explicit matching-rules table added to section 3. The classification mechanics themselves: no change (BRD v1.0 section 3, system action 2).</t>
+          <t>BRD v1.1: employer search-and-select added to the edit section (screen SC3 updated); matching rules documented. Classification mechanics: no change — Day-1 logic, BRD v1.0 section 3.</t>
         </is>
       </c>
     </row>
@@ -548,17 +540,17 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Already satisfied in substance — the design is validation-first: a manually typed name can never by itself establish ALOC; the classification results only from the independent system match against the approved Empaneled Company List (BRD v1.0 section 3, action 2; SC5 shows the re-classified result with match score). New: a supporting-evidence reference captured with the amendment; system-side EFR / document validation would be a new integration and is not proposed for this scope.</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>The design already works exactly this way. A name entered by the Credit user can never, by itself, establish a more favourable classification: the ALOC result is produced only by the system's independent match against the approved Empaneled Company List — if the corrected name does not match a listed, active employer, the application remains N-ALOC. This is the Day-1 classification model and this feature does not change it (BRD section 3; the match result including confidence score is displayed on screen SC5). Validation against EFR, salary records or employment documents is the Credit review that already takes place in the queue, where these documents are available to the user; an automated document-validation service is a separate initiative and not part of this change.</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>No change</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>BRD v1.1: validation-first principle stated verbatim + evidence-reference field. Classification independence: no change (already v1.0).</t>
+          <t>Already covered — BRD v1.0 section 3 (system action 2), SC5. No system change required.</t>
         </is>
       </c>
     </row>
@@ -572,17 +564,17 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>PUSH BACK. Consistent platform behaviour: none of the live Credit Queue Edit sections (Finalized Income, Liability Info, Length of Service, Other Income and Expenses) carries a reason field, and the amendment cannot of itself improve the classification (see item 2) — the control value of a reason code is limited while the full old-to-new trail, user and timestamp are already recorded in the Application History (BRD v1.0 section 3 action 6, SC6). A reason code adds friction to every correction without changing any system decision.</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>No — pushed back</t>
+          <t>We recommend keeping this edit consistent with the established Edit framework of the Credit Queue: none of the live edit functions (Finalized Income, Liability Information, Length of Service, Other Income and Expenses) captures a reason code, and the full old-to-new change, the user and the timestamp are already recorded in the Application History for every amendment (BRD section 3, screen SC6). Because the classification is system-derived (item 2), a reason code does not alter any decision outcome — it adds an input step to every correction. If the Bank sees value in reason codes, we suggest assessing it once, as a platform-wide convention across all Edit functions, rather than introducing it for this field alone.</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Not incorporated</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>No change to BRD. Fallback if insisted: reason dropdown is small development — can be added in v1.1 without redesign.</t>
+          <t>Traceability already covered — BRD v1.0 section 3 action 6, SC6. Reason-code convention: to be assessed as a platform-wide topic if prioritised.</t>
         </is>
       </c>
     </row>
@@ -599,17 +591,17 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>NOT IN SCOPE of this feature. This feature delivers the capability to edit the Employer Name and re-run the existing logic (classification, recalculation, Rule Engine, routing) — which is exactly the STP leg he describes, already in BRD v1.0 sections 3 and 6. A Controlled-STP / Exception decision matrix with delegated-authority routing is a broader credit-workflow design to be discussed as a new scope, not inside this change. Note the edit already happens inside the manual Credit Queue, operated by authorised Credit users under the existing L1/L2/L3 authority model.</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>No — new scope</t>
+          <t>The STP leg described is precisely what this feature delivers: a successfully matched employer automatically triggers re-classification, recalculation, Rule Engine re-run and routing with no further manual step (BRD sections 3 and 6). Equally important, this edit is not an unattended process — it is performed by an authorised Credit user inside the Credit Queue, which is itself the Bank's manual-review control layer with its L1/L2/L3 structure; an unmatched name simply remains N-ALOC. A Controlled-STP / Exception decision matrix with delegated-authority routing is a credit-workflow design that goes beyond the capability this change delivers (edit the employer name and re-run the existing decisioning). We suggest taking it up as its own initiative where it can be designed across all queue actions, not only this field.</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Not incorporated — new scope</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>STP leg: no change (v1.0 flow diagram + sections 3, 6). Decision matrix / authority routing: separate scope discussion.</t>
+          <t>STP behaviour: already in BRD v1.0 (flow + sections 3, 6). Decision matrix / delegated authority: proposed as a separate scope discussion.</t>
         </is>
       </c>
     </row>
@@ -623,17 +615,17 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>NOT IN SCOPE of this feature — belongs to the same new-scope discussion as item 4. All seven values are already recalculated and displayed to the Credit user after the re-run (ALOC with match score, category, Rule Engine Result, Approve Limit Result — BRD v1.0 sections 3-4, SC5), and the before/after record is in the Application History (SC6). Automated favourable-delta detection with approval gating is new control logic for the new scope.</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>No — new scope</t>
+          <t>Visibility is already there: after the re-run the Credit user sees the re-classified ALOC with its match score, the employer category, the refreshed Rule Engine Result and the recalculated Approve Limit Result on the same screen (BRD section 4, screen SC5), and the before/after record in the Application History (SC6) — so every one of the listed movements is visible to the deciding user before any decision is taken. Automated detection of a favourable delta with approval gating belongs to the same decision-matrix design as item 4 and we propose handling both in that separate initiative.</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Not incorporated — new scope</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Visibility of recalculated results: no change (v1.0 SC5/SC6). Impact-detection control: new scope with item 4.</t>
+          <t>Visibility of all recalculated values: already covered — BRD v1.0 sections 3-4, SC5/SC6. Delta-detection control: with item 4 in the new scope.</t>
         </is>
       </c>
     </row>
@@ -649,17 +641,17 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>PUSH BACK. Repeat edits are already bounded and fully visible: every edit re-runs the Rule Engine under the existing shared re-run counter — more than 2 Rule Engine failures auto-rejects the application (BRD v1.0 section 3 action 4) — and every edit writes its own Edit Information step with the full old-to-new trail (SC6). The edit is performed by authorised Credit users inside the controlled queue; additional authority for repeats belongs to the item 4 new-scope discussion if pursued.</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>No — pushed back</t>
+          <t>Repeat amendments are already bounded and visible by design. Every amendment re-runs the Rule Engine under the platform's shared re-run counter — an application that fails the Rule Engine more than twice is automatically rejected — and every amendment writes its own fully detailed step in the Application History (BRD section 3, SC6), so repeated activity is immediately visible to anyone reviewing the case. The action is restricted to authorised Credit users inside the controlled queue environment. A configurable repeat-amendment threshold with escalating authority is workable, but it belongs to the same authority-matrix design as item 4; we propose deciding it there so the rule is consistent across all queue edits.</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Not incorporated</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>No change to BRD (v1.0 already documents counter + per-edit audit). Fallback: configurable repeat threshold is feasible if the bank insists.</t>
+          <t>Bounding and traceability already covered — BRD v1.0 section 3 (re-run counter, per-edit audit), SC6. Configurable threshold: with the item 4 scope discussion.</t>
         </is>
       </c>
     </row>
@@ -672,17 +664,17 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Agreed — this is already the behaviour: the counter counts business Rule Engine failures of the application (existing platform rule, unchanged by this feature); technical/integration failures follow error handling and never consume the counter or reject the customer. One clarification sentence added so it is explicit.</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
+          <t>Confirmed — this is the existing behaviour. The counter counts business Rule Engine outcomes of the application; technical and integration failures are handled by the platform's error-handling and retry mechanisms and do not consume the counter or reject the customer. This is Day-1 platform behaviour that this feature re-uses unchanged; we will state it explicitly in the BRD for clarity.</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>No change</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>BRD v1.0 section 3 action 4 (existing shared counter); v1.1 adds one clarification sentence only.</t>
+          <t>Existing platform behaviour — BRD v1.0 section 3 action 4; one clarification sentence added in v1.1.</t>
         </is>
       </c>
     </row>
@@ -697,17 +689,17 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>The treatment is documented in BRD v1.0 section 5: no re-screening on the edit — consistent with every existing Edit section — and the corrected name reaches the screening system through the post-decision CIF-update call. Confirmation to be obtained from Compliance; the documented logic stands unless Compliance directs otherwise.</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
+          <t>The treatment is documented in the BRD (section 5) and is consistent with every existing edit function on the platform: screening is not re-triggered by a queue edit, and the corrected employer name reaches the screening system through the standard post-decision customer-update flow, so the screening record always carries the finalized value. We will take the action to put this in front of Compliance for confirmation; the documented logic stands unless Compliance directs otherwise.</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>No change</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>BRD v1.0 section 5 (EastNets row). Action: Compliance confirmation — owner Compliance; v1.1 adds a 'confirmed by Compliance on [date]' placeholder only.</t>
+          <t>Documented in BRD v1.0 section 5. Action: Compliance confirmation — placeholder for the confirmation date added in v1.1.</t>
         </is>
       </c>
     </row>
@@ -721,17 +713,17 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>PUSH BACK on new framework scope. Every data point listed is already captured per edit in the audit trail / Application History (user, timestamps, old/new name and classification — BRD v1.0 section 3 action 6, SC6) and is extractable for monitoring from day one. A dedicated fraud-monitoring capability / dashboards is reporting scope to be planned with item 18, not part of this change.</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>No — new scope</t>
+          <t>Every data point on this list is captured by the system today: each amendment is recorded in the audit trail and Application History with the user, timestamps and the old and new values of name and classification (BRD section 3, SC6), so amendment counts, user activity, classification changes and repeat patterns are all available for extraction from day one. Building fraud-monitoring views on top of that data is part of the Bank's control and reporting framework, which spans all portal activity — it is not specific to this feature and we propose planning it together with the reporting scope of item 18.</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Not incorporated — separate stream</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Monitoring source data: no change (v1.0 audit trail). Monitoring reports: new scope with item 18.</t>
+          <t>Monitoring source data: already covered — BRD v1.0 audit trail (section 3, SC6). Monitoring views: Bank reporting/control stream, with item 18.</t>
         </is>
       </c>
     </row>
@@ -746,17 +738,17 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Out of this feature — the Empaneled Company List is a bank-owned master that exists today with its own upload and maintenance process; its governance, data model and maker-checker are a separate change request. This feature consumes the master as-is and automatically inherits every improvement made to it.</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>No — separate CR</t>
+          <t>The Empaneled Company List is a Bank-owned master with its own established upload and maintenance process on the platform; its governance model, data dictionary and maker-checker controls are a standing capability question that applies to every function consuming the list, not only this one. We recommend raising it as a dedicated change request. This feature consumes the master as-is and will automatically benefit from any enrichment (aliases, Arabic names, employer IDs) made there.</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Not incorporated — separate CR</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Referenced in BRD dependencies only. Alias/Arabic matching quality (item 1) depends on this stream.</t>
+          <t>Out of this feature. Referenced in the BRD dependencies; matching quality of item 1 improves automatically with this stream.</t>
         </is>
       </c>
     </row>
@@ -771,17 +763,17 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Already covered: the four values exist as distinct, never-overwritten data points — customer-declared (Customer Journey input, never modified), system-derived original (kept at first edit), finalized working value, credit-amended (Source = Credit Department with Updated By/On) — BRD v1.0 section 3 action 1 and section 4; visible in SC5 (Company Name Source row). The finalized value is the single value used for the credit decision (section 5).</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
+          <t>This distinction exists by design and is preserved by this feature. The customer-declared name (journey input) and the government-record sponsor name are never modified; the system-derived original is retained from the first amendment onward; the finalized value carries an explicit source attribute (government record / customer journey / Credit Department) with the amending user and timestamp; and it is the finalized value, alone, that drives the credit decision and every downstream consumer (BRD sections 3, 4 and 5; visible on screen SC5). We will add a one-glance hierarchy table to the BRD so this is readable in a single place.</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>No change</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>BRD v1.0 sections 3, 4, 5 + SC5. v1.1 adds only a one-glance hierarchy table naming the same values.</t>
+          <t>Already covered — BRD v1.0 sections 3/4/5, SC5. v1.1 adds a summary table only (presentation, not scope).</t>
         </is>
       </c>
     </row>
@@ -794,17 +786,17 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Accepted — Development (small). Baseline already records old/new name, old source, old/new ALOC, user and timestamps on labelled lines (BRD v1.0 section 3 action 6, SC6). Extension adds employer ID, DBR, multiplier, limit, evidence reference, Rule Engine version and re-evaluation result — all values the re-run already produces. (Reason field follows the item 3 outcome.)</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>The complete picture is already recorded across the Application History. The Edit Information step captures the old and new employer name with the previous source and the old and new classification, with user and timestamps; the financial effects are then recorded by the existing system steps of the same run — recalculation, Rule Engine execution and result, and Limit Assignment with the recalculated limit (BRD section 3, screen SC6). The Rule Engine itself maintains version control of the published strategies, so the version evaluated is traceable. Duplicating the financial values inside one consolidated step is a presentation preference rather than a control gap; we recommend keeping the established step model that the whole platform audit follows.</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>No change</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>BRD v1.1: audit field list expanded; SC6 re-rendered. Base trail: no change (v1.0).</t>
+          <t>Already covered across the history steps — BRD v1.0 section 3 action 6 + system steps, SC6. Reason/evidence fields follow the item 3 outcome.</t>
         </is>
       </c>
     </row>
@@ -819,17 +811,17 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Accepted — his highlighted transaction paragraph is adopted verbatim. Locking during the run already exists (BRD v1.0 section 3 action 7); v1.1 makes the one-controlled-transaction / no-partial-commit / rollback-or-recovery rule explicit.</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>This reflects how the platform processes every queue edit today: the amendment and its downstream re-runs execute as one orchestrated flow while the application is locked against any other action, and the updated values are presented together on completion (BRD section 3). Transaction integrity and recovery behaviour are part of the platform's Day-1 processing architecture that all functions share — they are not introduced or altered by this feature. We will reflect the controlled-transaction statement in the BRD for clarity, with no change to scope.</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>No change</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>BRD v1.1: atomic-transaction clause in section 3; recovery status defined with item 15. Locking: no change (v1.0 action 7).</t>
+          <t>Platform processing model — BRD v1.0 section 3 action 7 (locking). v1.1 quotes the controlled-transaction statement for clarity only.</t>
         </is>
       </c>
     </row>
@@ -842,17 +834,17 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Already covered in principle: the application is locked during processing and a concurrent action gets 'The Application is in another request processing.' (BRD v1.0 section 3 action 7). v1.1 adds the stale-session / version-check wording.</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
+          <t>Covered by the existing locking model: while an amendment is processing the application is locked and any other user action receives 'The Application is in another request processing.' (BRD section 3). Session and version management are platform-level mechanisms common to all portal functions. We will add the stale-session wording to the BRD for completeness; no system change arises from this feature.</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>No change</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>BRD v1.0 section 3 action 7; v1.1 adds one strengthening sentence (version validation before save).</t>
+          <t>Already covered — BRD v1.0 section 3 action 7; v1.1 adds one completeness sentence.</t>
         </is>
       </c>
     </row>
@@ -866,17 +858,17 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Accepted — new non-functional section covering the listed failure modes, idempotency and recovery; pairs with items 7 and 13 (technical failures never consume the business counter; no partial state).</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>These are non-functional, platform-level requirements rather than requirements of this feature. Service failure handling, timeouts, retries, idempotency and recovery are governed by the platform's Day-1 architecture and apply uniformly to every function that calls the classification service, the Rule Engine or any integration — this feature introduces no new integration pattern; it re-uses the same services through the same error-handling framework. Defining or amending the resiliency standard is therefore an architecture-level topic, not a BRD item for this change.</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Not incorporated — platform NFR</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>BRD v1.1: new 'Failure handling and resiliency' section; engineering to size.</t>
+          <t>Governed by the Day-1 platform architecture; this feature adds no new integration pattern. No change to the BRD.</t>
         </is>
       </c>
     </row>
@@ -890,17 +882,17 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Already covered — this is exactly BRD v1.0 section 5: every consumer (application views across all queues and enquiry, CAM, Affordability Assessment Form, document stack, core banking, screening) reads the single finalized value after the update. The explicit one-sentence requirement is added above the table.</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
+          <t>This is already an explicit design principle of the BRD: section 5 lists every downstream consumer — the application views across all queues and enquiry, the CAM report, the Affordability Assessment Form, the document stack, core banking and screening — and each one reads the single finalized value after a successful update. There is one source of truth by construction. We will add the one-sentence requirement above the table so it reads as a rule as well as a mapping.</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>No change</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>BRD v1.0 section 5 (downstream consumers table); v1.1 adds the one-sentence explicit requirement only.</t>
+          <t>Already covered — BRD v1.0 section 5; v1.1 adds the one-sentence statement only.</t>
         </is>
       </c>
     </row>
@@ -915,17 +907,17 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Agreed by Head of Retail — already the design: the Application Form stays the customer's OTP-time record and the Customer Journey input is never modified (BRD v1.0 sections 3 and 5); the Customer-Declared vs Bank-Validated distinction is carried by the source data points of item 11.</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
+          <t>Noted with thanks — this is the current design. The Application Form permanently retains the customer's submission, the customer journey input is never modified by the amendment, and the distinction requested is exactly the source attribution of item 11. We will adopt the terminology 'Customer Declared Employer / Bank Validated Employer' in the source table.</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>No change</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>BRD v1.0 sections 3, 5; v1.1 adopts the 'Customer Declared / Bank Validated' terminology in the item 11 table.</t>
+          <t>Already covered — BRD v1.0 sections 3 and 5; terminology adopted in the item 11 table.</t>
         </is>
       </c>
     </row>
@@ -938,17 +930,17 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>PUSH BACK on scope. The reporting dataset is derivable from the enhanced audit trail (item 12) from day one; a dedicated MIS / report pack is reporting scope to be planned separately together with item 9 — not part of this change. STP/exception percentages additionally depend on the item 4 new-scope decision matrix.</t>
-        </is>
-      </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>No — new scope</t>
+          <t>As with item 9, the underlying data for this reporting is produced by the feature from day one through the audit trail and Application History. Management reporting itself is a platform reporting capability that serves all functions and is planned as its own stream — we recommend consolidating the item 9 and item 18 requirements into one reporting scope there. The STP/exception percentages additionally presuppose the decision matrix of item 4, so they follow that discussion.</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Not incorporated — separate stream</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Source dataset: covered by items 12 / v1.0 audit trail. Report delivery: separate reporting scope with item 9.</t>
+          <t>Source data covered (BRD v1.0 audit trail). Report delivery: Bank reporting stream together with item 9.</t>
         </is>
       </c>
     </row>
@@ -962,17 +954,17 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Partially accepted. The validation-first principle and the one-controlled-transaction paragraph are adopted (items 2 and 13 — the first is already how classification works, the second is made explicit). The exception-routing clause (material positive impact / repeated amendment -&gt; control queue) follows the items 4-6 outcome — new scope / pushed back as above.</t>
-        </is>
-      </c>
-      <c r="C20" s="6" t="inlineStr">
-        <is>
-          <t>Partial</t>
+          <t>Both principles are restatements of how the platform behaves today. Manual amendment cannot establish eligibility or classification — the system validates independently against the Empaneled Company List before anything recalculates (item 2), successful validation flows straight through (item 4), and an unverified employer simply remains N-ALOC within the controlled queue. The processing model is one orchestrated, locked flow (item 13). The additional exception-routing conditions (material impact, repeated amendment) belong to the decision-matrix initiative of item 4. We will reflect the two principles in the BRD wording; they confirm the design rather than change it.</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>No change</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Validation-first + atomic transaction: in v1.1. Exception-routing clause: follows the item 4 new-scope discussion.</t>
+          <t>Both paragraphs reflected as confirming statements in v1.1; exception-routing conditions follow the item 4 initiative.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
RF-3309: feedback matrix v4 — highlighted requirements to v1.1; BRD evidence column with screens/pages
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DpzepkLYwCzujeEtvjJxcF
</commit_message>
<xml_diff>
--- a/docs/brd/RF-3309/RF-3309_HoR_feedback_matrix.xlsx
+++ b/docs/brd/RF-3309/RF-3309_HoR_feedback_matrix.xlsx
@@ -90,7 +90,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -101,6 +101,7 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -181,6 +182,436 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2800350" cy="2047875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2800350" cy="2047875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3638550" cy="2047875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3810000" cy="1409700"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Image 4" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>5</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2800350" cy="2047875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="5" name="Image 5" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>6</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3638550" cy="2047875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="6" name="Image 6" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1447800" cy="2047875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="7" name="Image 7" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId7"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>8</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1447800" cy="2047875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="8" name="Image 8" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId8"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>9</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3638550" cy="2047875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="9" name="Image 9" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId9"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>11</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2800350" cy="2047875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="10" name="Image 10" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId10"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>12</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3638550" cy="2047875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="11" name="Image 11" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId11"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>13</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1447800" cy="2047875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="12" name="Image 12" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId12"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>14</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1447800" cy="2047875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="13" name="Image 13" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId13"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>16</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1447800" cy="2047875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="14" name="Image 14" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId14"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>17</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1447800" cy="2047875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="15" name="Image 15" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId15"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>18</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3638550" cy="2047875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="16" name="Image 16" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId16"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>19</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1447800" cy="2047875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="17" name="Image 17" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId17"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -472,13 +903,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="56" customWidth="1" min="1" max="1"/>
-    <col width="66" customWidth="1" min="2" max="2"/>
-    <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="56" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -502,15 +935,22 @@
           <t>Note / description</t>
         </is>
       </c>
-    </row>
-    <row r="2">
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>BRD reference</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Evidence (BRD v1.0 screen / page)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="222" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>1. Employer selection and validation
-The Employer Name should not operate as an unrestricted free-text field wherever this can be avoided. The preferred design should allow the Credit user to search and select the employer from the approved Employer Master / Empaneled Company List.
-If free text amendment is required as an exception, the system should require additional validation before the updated employer can affect ALOC, DBR, income multiplier, eligibility or limit.
-Please also define the employer matching logic, including Such as Exact match, Fuzzy match / confidence threshold., Arabic and English employer names, Trade name versus legal name, Employer aliases, Duplicate employer records, Active/inactive employer status.
-The BRD currently states that the updated name will be matched against the Empaneled Company List and the classification rerun. This needs to be more explicitly controlled</t>
+The Employer Name should not operate as an unrestricted free-text field wherever this can be avoided. The preferred design should allow the Credit user to search and select the employer from the approved Employer Master / Empaneled Company List. If free text amendment is required as an exception, the system should require additional validation before the updated employer can affect ALOC, DBR, income multiplier, eligibility or limit. Please also define the employer matching logic, including Such as Exact match, Fuzzy match / confidence threshold., Arabic and English employer names, Trade name versus legal name, Employer aliases, Duplicate employer records, Active/inactive employer status. The BRD currently states that the updated name will be matched against the Empaneled Company List and the classification rerun. This needs to be more explicitly controlled</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -528,14 +968,18 @@
           <t>BRD v1.1: employer search-and-select added to the edit section (screen SC3 updated); matching rules documented. Classification mechanics: no change — Day-1 logic, BRD v1.0 section 3.</t>
         </is>
       </c>
-    </row>
-    <row r="3">
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>BRD section 2 — Edit Application pop-up (screen SC3; to be updated with the employer picker in v1.1)</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr"/>
+    </row>
+    <row r="3" ht="170" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>2. Source validation before applying the amendment
-The employer amendment should follow a validation-first model.
-Where available, the amended employer should be validated against the relevant authoritative or supporting source, such as EFR / government employment record, salary information, employment certificate, pays lip or any other approved source used by the Bank.
-A manual amendment by the Credit user should not, by itself, be sufficient to establish a more favorable employer classification.</t>
+The employer amendment should follow a validation-first model. Where available, the amended employer should be validated against the relevant authoritative or supporting source, such as EFR / government employment record, salary information, employment certificate, pays lip or any other approved source used by the Bank. A manual amendment by the Credit user should not, by itself, be sufficient to establish a more favorable employer classification.</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -543,7 +987,7 @@
           <t>The design already works exactly this way. A name entered by the Credit user can never, by itself, establish a more favourable classification: the ALOC result is produced only by the system's independent match against the approved Empaneled Company List — if the corrected name does not match a listed, active employer, the application remains N-ALOC. This is the Day-1 classification model and this feature does not change it (BRD section 3; the match result including confidence score is displayed on screen SC5). Validation against EFR, salary records or employment documents is the Credit review that already takes place in the queue, where these documents are available to the user; an automated document-validation service is a separate initiative and not part of this change.</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="5" t="inlineStr">
         <is>
           <t>No change</t>
         </is>
@@ -553,13 +997,18 @@
           <t>Already covered — BRD v1.0 section 3 (system action 2), SC5. No system change required.</t>
         </is>
       </c>
-    </row>
-    <row r="4">
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>BRD section 3 (system action 2) and section 4 — screen SC5: ALOC shown with the independent match score</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr"/>
+    </row>
+    <row r="4" ht="170" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>3. Mandatory reason for change
-Every Employer Name amendment must require a mandatory reason code.
-Suggested reasons: Spelling correction, Employer legal name / trade name correction, Employer alias, EFR / government record mismatch, Employer Master mapping issue, Customer-provided information correction &amp; Other. (If Other is selected, a mandatory comment should be required)</t>
+Every Employer Name amendment must require a mandatory reason code. Suggested reasons: Spelling correction, Employer legal name / trade name correction, Employer alias, EFR / government record mismatch, Employer Master mapping issue, Customer-provided information correction &amp; Other. (If Other is selected, a mandatory comment should be required)</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -567,7 +1016,7 @@
           <t>We recommend keeping this edit consistent with the established Edit framework of the Credit Queue: none of the live edit functions (Finalized Income, Liability Information, Length of Service, Other Income and Expenses) captures a reason code, and the full old-to-new change, the user and the timestamp are already recorded in the Application History for every amendment (BRD section 3, screen SC6). Because the classification is system-derived (item 2), a reason code does not alter any decision outcome — it adds an input step to every correction. If the Bank sees value in reason codes, we suggest assessing it once, as a platform-wide convention across all Edit functions, rather than introducing it for this field alone.</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>Not incorporated</t>
         </is>
@@ -577,16 +1026,18 @@
           <t>Traceability already covered — BRD v1.0 section 3 action 6, SC6. Reason-code convention: to be assessed as a platform-wide topic if prioritised.</t>
         </is>
       </c>
-    </row>
-    <row r="5">
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>BRD section 3 (system action 6) — Application History records every amendment (screen SC6)</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr"/>
+    </row>
+    <row r="5" ht="198" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>4. STP versus exception handling
-Please define a clear STP decision matrix.
-The expected design should be:
-STP: Employer successfully matched and validated, no conflicting information and no exception criteria triggered -&gt; automatically update the employer, rerun classification, recalculation, Rule Engine and routing.
-Controlled STP: Employer is validated, but the amendment creates a material positive credit impact -&gt; system performs the recalculation automatically but applies the relevant Credit approval level / delegated authority.
-Exception: Employer cannot be confidently matched, evidence conflicts, repeated amendments are detected, or other risk conditions are triggered -&gt; application should move to manual review rather than allowing an unrestricted override.</t>
+Please define a clear STP decision matrix. The expected design should be: STP: Employer successfully matched and validated, no conflicting information and no exception criteria triggered -&gt; automatically update the employer, rerun classification, recalculation, Rule Engine and routing. Controlled STP: Employer is validated, but the amendment creates a material positive credit impact -&gt; system performs the recalculation automatically but applies the relevant Credit approval level / delegated authority. Exception: Employer cannot be confidently matched, evidence conflicts, repeated amendments are detected, or other risk conditions are triggered -&gt; application should move to manual review rather than allowing an unrestricted override.</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -594,7 +1045,7 @@
           <t>The STP leg described is precisely what this feature delivers: a successfully matched employer automatically triggers re-classification, recalculation, Rule Engine re-run and routing with no further manual step (BRD sections 3 and 6). Equally important, this edit is not an unattended process — it is performed by an authorised Credit user inside the Credit Queue, which is itself the Bank's manual-review control layer with its L1/L2/L3 structure; an unmatched name simply remains N-ALOC. A Controlled-STP / Exception decision matrix with delegated-authority routing is a credit-workflow design that goes beyond the capability this change delivers (edit the employer name and re-run the existing decisioning). We suggest taking it up as its own initiative where it can be designed across all queue actions, not only this field.</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>Not incorporated — new scope</t>
         </is>
@@ -604,13 +1055,18 @@
           <t>STP behaviour: already in BRD v1.0 (flow + sections 3, 6). Decision matrix / delegated authority: proposed as a separate scope discussion.</t>
         </is>
       </c>
-    </row>
-    <row r="6">
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>BRD end-to-end flow + sections 3 and 6 — the STP leg as built</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr"/>
+    </row>
+    <row r="6" ht="170" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>5. Material positive credit impact
-The system must identify whenever the employer amendment creates a more favorable credit position, including where it: Changes N-ALOC to ALOC. Moves the employer into a more favorable category. Increases permitted DBR. Increases income multiplier. Increases approved/proposed limit. Removes a deviation. Converts an otherwise ineligible application into an eligible application.
-These cases should be specifically controlled and visible to the approving Credit user.</t>
+The system must identify whenever the employer amendment creates a more favorable credit position, including where it: Changes N-ALOC to ALOC. Moves the employer into a more favorable category. Increases permitted DBR. Increases income multiplier. Increases approved/proposed limit. Removes a deviation. Converts an otherwise ineligible application into an eligible application. These cases should be specifically controlled and visible to the approving Credit user.</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -618,7 +1074,7 @@
           <t>Visibility is already there: after the re-run the Credit user sees the re-classified ALOC with its match score, the employer category, the refreshed Rule Engine Result and the recalculated Approve Limit Result on the same screen (BRD section 4, screen SC5), and the before/after record in the Application History (SC6) — so every one of the listed movements is visible to the deciding user before any decision is taken. Automated detection of a favourable delta with approval gating belongs to the same decision-matrix design as item 4 and we propose handling both in that separate initiative.</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>Not incorporated — new scope</t>
         </is>
@@ -628,15 +1084,18 @@
           <t>Visibility of all recalculated values: already covered — BRD v1.0 sections 3-4, SC5/SC6. Delta-detection control: with item 4 in the new scope.</t>
         </is>
       </c>
-    </row>
-    <row r="7">
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>BRD sections 3–4 — screen SC5: re-classified ALOC, Rule Engine Result and Approve Limit Result visible to the deciding user</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr"/>
+    </row>
+    <row r="7" ht="170" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>6. Repeat employer amendments
-The current BRD states that there is no cap on repeat edits.
-Please revise this requirement.
-Unlimited employer amendments are not recommended where the employer classification directly impacts DBR, multiplier and limit assignment.
-The system should have a configurable control over repeat amendments. At minimum, any subsequent amendment after the initial correction should trigger additional authority, reason capture and appropriate monitoring.</t>
+The current BRD states that there is no cap on repeat edits. Please revise this requirement. Unlimited employer amendments are not recommended where the employer classification directly impacts DBR, multiplier and limit assignment. The system should have a configurable control over repeat amendments. At minimum, any subsequent amendment after the initial correction should trigger additional authority, reason capture and appropriate monitoring.</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -644,7 +1103,7 @@
           <t>Repeat amendments are already bounded and visible by design. Every amendment re-runs the Rule Engine under the platform's shared re-run counter — an application that fails the Rule Engine more than twice is automatically rejected — and every amendment writes its own fully detailed step in the Application History (BRD section 3, SC6), so repeated activity is immediately visible to anyone reviewing the case. The action is restricted to authorised Credit users inside the controlled queue environment. A configurable repeat-amendment threshold with escalating authority is workable, but it belongs to the same authority-matrix design as item 4; we propose deciding it there so the rule is consistent across all queue edits.</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>Not incorporated</t>
         </is>
@@ -654,8 +1113,14 @@
           <t>Bounding and traceability already covered — BRD v1.0 section 3 (re-run counter, per-edit audit), SC6. Configurable threshold: with the item 4 scope discussion.</t>
         </is>
       </c>
-    </row>
-    <row r="8">
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>BRD section 3 (re-run counter) — per-edit history steps (screen SC6)</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr"/>
+    </row>
+    <row r="8" ht="170" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>7. Rule Engine rerun counter
@@ -667,7 +1132,7 @@
           <t>Confirmed — this is the existing behaviour. The counter counts business Rule Engine outcomes of the application; technical and integration failures are handled by the platform's error-handling and retry mechanisms and do not consume the counter or reject the customer. This is Day-1 platform behaviour that this feature re-uses unchanged; we will state it explicitly in the BRD for clarity.</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>No change</t>
         </is>
@@ -677,14 +1142,18 @@
           <t>Existing platform behaviour — BRD v1.0 section 3 action 4; one clarification sentence added in v1.1.</t>
         </is>
       </c>
-    </row>
-    <row r="9">
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>BRD section 3, system actions table (action 4 — Rule Engine re-run and counter)</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr"/>
+    </row>
+    <row r="9" ht="170" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
           <t>8. AML / KYC impact
-The BRD currently states that AML screening will not be rerun following an employer amendment.
-Please reconfirm this treatment with Compliance and clearly document the agreed logic.
-If employer information forms part of customer risk assessment, KYC profiling or screening, the appropriate refresh/reassessment should be triggered.</t>
+The BRD currently states that AML screening will not be rerun following an employer amendment. Please reconfirm this treatment with Compliance and clearly document the agreed logic. If employer information forms part of customer risk assessment, KYC profiling or screening, the appropriate refresh/reassessment should be triggered.</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -692,7 +1161,7 @@
           <t>The treatment is documented in the BRD (section 5) and is consistent with every existing edit function on the platform: screening is not re-triggered by a queue edit, and the corrected employer name reaches the screening system through the standard post-decision customer-update flow, so the screening record always carries the finalized value. We will take the action to put this in front of Compliance for confirmation; the documented logic stands unless Compliance directs otherwise.</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>No change</t>
         </is>
@@ -702,13 +1171,18 @@
           <t>Documented in BRD v1.0 section 5. Action: Compliance confirmation — placeholder for the confirmation date added in v1.1.</t>
         </is>
       </c>
-    </row>
-    <row r="10">
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>BRD section 5 — downstream consumers table, AML screening row</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr"/>
+    </row>
+    <row r="10" ht="170" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
           <t>9. Fraud monitoring
-Please include employer amendments in the fraud/control monitoring framework.
-At minimum, the system should make available for monitoring Number of employer amendments per application, Amendments by Credit user, N-ALOC to ALOC changes, Employer-category upgrades, Resulting limit increases, Repeated amendment to the same employers, Unusual concentration of amendments by a particular user.</t>
+Please include employer amendments in the fraud/control monitoring framework. At minimum, the system should make available for monitoring Number of employer amendments per application, Amendments by Credit user, N-ALOC to ALOC changes, Employer-category upgrades, Resulting limit increases, Repeated amendment to the same employers, Unusual concentration of amendments by a particular user.</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -716,7 +1190,7 @@
           <t>Every data point on this list is captured by the system today: each amendment is recorded in the audit trail and Application History with the user, timestamps and the old and new values of name and classification (BRD section 3, SC6), so amendment counts, user activity, classification changes and repeat patterns are all available for extraction from day one. Building fraud-monitoring views on top of that data is part of the Bank's control and reporting framework, which spans all portal activity — it is not specific to this feature and we propose planning it together with the reporting scope of item 18.</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>Not incorporated — separate stream</t>
         </is>
@@ -726,14 +1200,18 @@
           <t>Monitoring source data: already covered — BRD v1.0 audit trail (section 3, SC6). Monitoring views: Bank reporting/control stream, with item 18.</t>
         </is>
       </c>
-    </row>
-    <row r="11">
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>BRD section 3 (action 6) — audit data available per amendment (screen SC6)</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr"/>
+    </row>
+    <row r="11" ht="170" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
           <t>10. Employer Master governance
-Please define the ownership and governance of the Employer Master / Empaneled Company List.
-This should cover Employer ID if available, Legal name, Trade name, Arabic/English names, Aliases, ALOC classification, Category, Industry/sector, Effective date and Active/inactive status.
-Maker-checker for employer-master changes.</t>
+Please define the ownership and governance of the Employer Master / Empaneled Company List. This should cover Employer ID if available, Legal name, Trade name, Arabic/English names, Aliases, ALOC classification, Category, Industry/sector, Effective date and Active/inactive status. Maker-checker for employer-master changes.</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -741,7 +1219,7 @@
           <t>The Empaneled Company List is a Bank-owned master with its own established upload and maintenance process on the platform; its governance model, data dictionary and maker-checker controls are a standing capability question that applies to every function consuming the list, not only this one. We recommend raising it as a dedicated change request. This feature consumes the master as-is and will automatically benefit from any enrichment (aliases, Arabic names, employer IDs) made there.</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>Not incorporated — separate CR</t>
         </is>
@@ -751,14 +1229,18 @@
           <t>Out of this feature. Referenced in the BRD dependencies; matching quality of item 1 improves automatically with this stream.</t>
         </is>
       </c>
-    </row>
-    <row r="12">
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Referenced in the BRD dependencies only (separate change request)</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr"/>
+    </row>
+    <row r="12" ht="170" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
           <t>11. Source hierarchy
-The BRD should clearly distinguish between Customer-declared Employer Name, Original system-derived Employer Name, Validated Employer Name and Credit-amended Employer Name.
-The original source should never be lost or overwritten.
-Please also define the source hierarchy so downstream users can clearly understand which employer information has been used for the final credit decision.</t>
+The BRD should clearly distinguish between Customer-declared Employer Name, Original system-derived Employer Name, Validated Employer Name and Credit-amended Employer Name. The original source should never be lost or overwritten. Please also define the source hierarchy so downstream users can clearly understand which employer information has been used for the final credit decision.</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -766,7 +1248,7 @@
           <t>This distinction exists by design and is preserved by this feature. The customer-declared name (journey input) and the government-record sponsor name are never modified; the system-derived original is retained from the first amendment onward; the finalized value carries an explicit source attribute (government record / customer journey / Credit Department) with the amending user and timestamp; and it is the finalized value, alone, that drives the credit decision and every downstream consumer (BRD sections 3, 4 and 5; visible on screen SC5). We will add a one-glance hierarchy table to the BRD so this is readable in a single place.</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C12" s="5" t="inlineStr">
         <is>
           <t>No change</t>
         </is>
@@ -776,8 +1258,14 @@
           <t>Already covered — BRD v1.0 sections 3/4/5, SC5. v1.1 adds a summary table only (presentation, not scope).</t>
         </is>
       </c>
-    </row>
-    <row r="13">
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>BRD sections 3/4/5 — screen SC5: Company Name Source attribution</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr"/>
+    </row>
+    <row r="13" ht="170" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
           <t>12. Enhanced audit trail
@@ -789,7 +1277,7 @@
           <t>The complete picture is already recorded across the Application History. The Edit Information step captures the old and new employer name with the previous source and the old and new classification, with user and timestamps; the financial effects are then recorded by the existing system steps of the same run — recalculation, Rule Engine execution and result, and Limit Assignment with the recalculated limit (BRD section 3, screen SC6). The Rule Engine itself maintains version control of the published strategies, so the version evaluated is traceable. Duplicating the financial values inside one consolidated step is a presentation preference rather than a control gap; we recommend keeping the established step model that the whole platform audit follows.</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C13" s="5" t="inlineStr">
         <is>
           <t>No change</t>
         </is>
@@ -799,14 +1287,18 @@
           <t>Already covered across the history steps — BRD v1.0 section 3 action 6 + system steps, SC6. Reason/evidence fields follow the item 3 outcome.</t>
         </is>
       </c>
-    </row>
-    <row r="14">
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>BRD section 3 — Edit Information step + system steps of the same run (screen SC6)</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr"/>
+    </row>
+    <row r="14" ht="170" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
           <t>13. Atomic processing / rollback
-All employer-related changes must be processed as one atomic transaction.
-The Employer Name should not be successfully updated while the classification, limit assignment or Rule Engine remains on the previous value.
-If any part of the recalculation or integration fails, the system should either Roll back completely to the last successful state; or Hold the application in a controlled pending/error status for recovery. Partial updates should not be permitted.</t>
+All employer-related changes must be processed as one atomic transaction. The Employer Name should not be successfully updated while the classification, limit assignment or Rule Engine remains on the previous value. If any part of the recalculation or integration fails, the system should either Roll back completely to the last successful state; or Hold the application in a controlled pending/error status for recovery. Partial updates should not be permitted.</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -814,7 +1306,7 @@
           <t>This reflects how the platform processes every queue edit today: the amendment and its downstream re-runs execute as one orchestrated flow while the application is locked against any other action, and the updated values are presented together on completion (BRD section 3). Transaction integrity and recovery behaviour are part of the platform's Day-1 processing architecture that all functions share — they are not introduced or altered by this feature. We will reflect the controlled-transaction statement in the BRD for clarity, with no change to scope.</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C14" s="5" t="inlineStr">
         <is>
           <t>No change</t>
         </is>
@@ -824,8 +1316,14 @@
           <t>Platform processing model — BRD v1.0 section 3 action 7 (locking). v1.1 quotes the controlled-transaction statement for clarity only.</t>
         </is>
       </c>
-    </row>
-    <row r="15">
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>BRD section 3 — system actions executed as one locked flow (action 7)</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr"/>
+    </row>
+    <row r="15" ht="170" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
           <t>14. Concurrency and locking
@@ -837,7 +1335,7 @@
           <t>Covered by the existing locking model: while an amendment is processing the application is locked and any other user action receives 'The Application is in another request processing.' (BRD section 3). Session and version management are platform-level mechanisms common to all portal functions. We will add the stale-session wording to the BRD for completeness; no system change arises from this feature.</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
         <is>
           <t>No change</t>
         </is>
@@ -847,13 +1345,18 @@
           <t>Already covered — BRD v1.0 section 3 action 7; v1.1 adds one completeness sentence.</t>
         </is>
       </c>
-    </row>
-    <row r="16">
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>BRD section 3, action 7 — locking / concurrent-action message</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr"/>
+    </row>
+    <row r="16" ht="170" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
           <t>15. Failure handling and resiliency
-Please add explicit handling for Employer-classification service failure, Rule Engine timeout, Integration/API timeout, Duplicate submission, Retry, Idempotency, Partial processing and Recovery/reconciliation.
-A technical failure should not leave the application in an inconsistent state.</t>
+Please add explicit handling for Employer-classification service failure, Rule Engine timeout, Integration/API timeout, Duplicate submission, Retry, Idempotency, Partial processing and Recovery/reconciliation. A technical failure should not leave the application in an inconsistent state.</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -861,7 +1364,7 @@
           <t>These are non-functional, platform-level requirements rather than requirements of this feature. Service failure handling, timeouts, retries, idempotency and recovery are governed by the platform's Day-1 architecture and apply uniformly to every function that calls the classification service, the Rule Engine or any integration — this feature introduces no new integration pattern; it re-uses the same services through the same error-handling framework. Defining or amending the resiliency standard is therefore an architecture-level topic, not a BRD item for this change.</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
         <is>
           <t>Not incorporated — platform NFR</t>
         </is>
@@ -871,13 +1374,18 @@
           <t>Governed by the Day-1 platform architecture; this feature adds no new integration pattern. No change to the BRD.</t>
         </is>
       </c>
-    </row>
-    <row r="17">
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Platform Day-1 architecture — no BRD item (non-functional standard)</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr"/>
+    </row>
+    <row r="17" ht="170" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
           <t>16. Downstream consistency
-Please add an explicit requirement that all downstream systems and documents must consume the same finalized Employer Name and classification following a successful update.
-There should be no situation where one system shows the original employer while another uses the amended employer for credit decisioning.</t>
+Please add an explicit requirement that all downstream systems and documents must consume the same finalized Employer Name and classification following a successful update. There should be no situation where one system shows the original employer while another uses the amended employer for credit decisioning.</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -885,7 +1393,7 @@
           <t>This is already an explicit design principle of the BRD: section 5 lists every downstream consumer — the application views across all queues and enquiry, the CAM report, the Affordability Assessment Form, the document stack, core banking and screening — and each one reads the single finalized value after a successful update. There is one source of truth by construction. We will add the one-sentence requirement above the table so it reads as a rule as well as a mapping.</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C17" s="5" t="inlineStr">
         <is>
           <t>No change</t>
         </is>
@@ -895,14 +1403,18 @@
           <t>Already covered — BRD v1.0 section 5; v1.1 adds the one-sentence statement only.</t>
         </is>
       </c>
-    </row>
-    <row r="18">
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>BRD section 5 — every consumer reads the single finalized value</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr"/>
+    </row>
+    <row r="18" ht="170" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
           <t>17. Customer-declared information
-I agree with the current approach that the original Application Form should continue to retain what the customer originally submitted.
-However, internally the system should clearly distinguish between: Customer Declared Employer and Bank Validated Employer.
-The customer declaration should never be overwritten.</t>
+I agree with the current approach that the original Application Form should continue to retain what the customer originally submitted. However, internally the system should clearly distinguish between: Customer Declared Employer and Bank Validated Employer. The customer declaration should never be overwritten.</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -910,7 +1422,7 @@
           <t>Noted with thanks — this is the current design. The Application Form permanently retains the customer's submission, the customer journey input is never modified by the amendment, and the distinction requested is exactly the source attribution of item 11. We will adopt the terminology 'Customer Declared Employer / Bank Validated Employer' in the source table.</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C18" s="5" t="inlineStr">
         <is>
           <t>No change</t>
         </is>
@@ -920,8 +1432,14 @@
           <t>Already covered — BRD v1.0 sections 3 and 5; terminology adopted in the item 11 table.</t>
         </is>
       </c>
-    </row>
-    <row r="19">
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>BRD sections 3 and 5 — Application Form retained; journey input never modified</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr"/>
+    </row>
+    <row r="19" ht="170" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
           <t>18. MIS and management reporting
@@ -933,7 +1451,7 @@
           <t>As with item 9, the underlying data for this reporting is produced by the feature from day one through the audit trail and Application History. Management reporting itself is a platform reporting capability that serves all functions and is planned as its own stream — we recommend consolidating the item 9 and item 18 requirements into one reporting scope there. The STP/exception percentages additionally presuppose the decision matrix of item 4, so they follow that discussion.</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="C19" s="6" t="inlineStr">
         <is>
           <t>Not incorporated — separate stream</t>
         </is>
@@ -943,32 +1461,44 @@
           <t>Source data covered (BRD v1.0 audit trail). Report delivery: Bank reporting stream together with item 9.</t>
         </is>
       </c>
-    </row>
-    <row r="20">
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Audit dataset produced from day one (screen SC6); reporting delivery separate</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr"/>
+    </row>
+    <row r="20" ht="222" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
           <t>Explicit requirements (highlighted paragraphs)
-Employer Name amendment shall follow a validation-first, exception-based model. Manual amendment shall not by itself establish employer eligibility or classification. The system shall independently validate the amended employer against approved Employer Master data [...] Where validation is successful and no exception criteria are triggered, processing shall continue STP. Where the amendment results in an unverified employer, ambiguous match, material positive credit impact, repeated amendment or conflicting source information, the application shall automatically route to the applicable control/approval queue.
-The Employer Name update, employer classification, calculated variables, limit assignment, Rule Engine execution and routing shall be treated as one controlled transaction. In case of any failure, no partial update shall be committed [...].</t>
+Employer Name amendment shall follow a validation-first, exception-based model. Manual amendment shall not by itself establish employer eligibility or classification. The system shall independently validate the amended employer against approved Employer Master data [...] Where validation is successful and no exception criteria are triggered, processing shall continue STP. Where the amendment results in an unverified employer, ambiguous match, material positive credit impact, repeated amendment or conflicting source information, the application shall automatically route to the applicable control/approval queue. The Employer Name update, employer classification, calculated variables, limit assignment, Rule Engine execution and routing shall be treated as one controlled transaction. In case of any failure, no partial update shall be committed [...].</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Both principles are restatements of how the platform behaves today. Manual amendment cannot establish eligibility or classification — the system validates independently against the Empaneled Company List before anything recalculates (item 2), successful validation flows straight through (item 4), and an unverified employer simply remains N-ALOC within the controlled queue. The processing model is one orchestrated, locked flow (item 13). The additional exception-routing conditions (material impact, repeated amendment) belong to the decision-matrix initiative of item 4. We will reflect the two principles in the BRD wording; they confirm the design rather than change it.</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>No change</t>
+          <t>Both principles are restatements of how the platform behaves today — manual amendment cannot establish eligibility or classification (the system validates independently against the Empaneled Company List before anything recalculates), successful validation flows straight through, an unverified employer remains N-ALOC within the controlled queue, and the processing executes as one orchestrated, locked flow. We will include both paragraphs in BRD v1.1 as governing statements; the additional exception-routing conditions (material positive impact, repeated amendment) follow the decision-matrix initiative of item 4.</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Both paragraphs reflected as confirming statements in v1.1; exception-routing conditions follow the item 4 initiative.</t>
-        </is>
-      </c>
+          <t>BRD v1.1: both paragraphs included as governing statements (feature overview + section 3). Exception-routing conditions: with the item 4 initiative.</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>BRD v1.1 — governing statements added to overview and section 3</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
RF-3309: align HoR feedback matrix with approved BRD V1.1
Re-verify every row against the final edited V1.1: item 1 updated to the
dropdown + Other/free-text design, items 6-7 reworded for the no-cap
re-run decision, highlighted requirements referenced to the matching
rules and controlled-transaction action. All not-incorporated rows now
read 'To be discussed' with the MVP 1.1 scope note.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DpzepkLYwCzujeEtvjJxcF
</commit_message>
<xml_diff>
--- a/docs/brd/RF-3309/RF-3309_HoR_feedback_matrix.xlsx
+++ b/docs/brd/RF-3309/RF-3309_HoR_feedback_matrix.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="HoR feedback matrix" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HoR feedback matrix" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -185,7 +185,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>5</col>
@@ -200,13 +200,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -225,13 +228,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -250,13 +256,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId3"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId3"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -275,13 +284,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId4"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId4"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -300,13 +312,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId5"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId5"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -325,13 +340,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId6"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId6"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -350,13 +368,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId7"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId7"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -375,13 +396,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId8"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId8"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -400,13 +424,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId9"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId9"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -425,13 +452,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId10"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId10"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -450,13 +480,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId11"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId11"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -475,13 +508,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId12"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId12"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -500,13 +536,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId13"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId13"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -525,13 +564,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId14"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId14"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -550,13 +592,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId15"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId15"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -575,13 +620,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId16"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId16"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -600,13 +648,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId17"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId17"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -955,7 +1006,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Agreed. The design will be updated so the Credit user searches and selects the employer from the Empaneled Company List, with free-text entry kept only as an exception path. One point of clarity: the matching and classification logic is not new to this feature — it is the Day-1 platform logic (name matching against the Empaneled Company List at a 90% confidence threshold, company category and active status checks), and the edit simply re-runs it. We will document these matching rules explicitly in the BRD. Coverage of aliases, Arabic names and duplicates is a function of the Empaneled Company List data itself and is addressed under item 10.</t>
+          <t>Agreed and incorporated. In the final V1.1 design the Company Name is a dropdown list sourced from the Empaneled Company List; where the employer is not in the list, the user selects 'Other' and enters the name as free text (customer-journey validation applies). The matching and classification logic is not new to this feature — it is the Day-1 platform logic (name matching against the Empaneled Company List at a 90% confidence threshold, company category and active status): classification is never taken from the typed text itself, and an employer with no confident match remains N-ALOC.</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -965,12 +1016,12 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>BRD v1.1: employer search-and-select added to the edit section (screen SC3 updated); matching rules documented. Classification mechanics: no change — Day-1 logic, BRD v1.0 section 3.</t>
+          <t>Incorporated in BRD V1.1: Company Name as dropdown over the Empaneled Company List with 'Other' → free text when not listed (section 2, SC3); employer matching rules documented. Classification mechanics unchanged — Day-1 logic, section 3.</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>BRD section 2 — Edit Application pop-up (screen SC3; to be updated with the employer picker in v1.1)</t>
+          <t>BRD V1.1 section 2 — Company Name field (dropdown + 'Other'/free text) and Employer matching rules table</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr"/>
@@ -1018,12 +1069,12 @@
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>Not incorporated</t>
+          <t>To be discussed</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Traceability already covered — BRD v1.0 section 3 action 6, SC6. Reason-code convention: to be assessed as a platform-wide topic if prioritised.</t>
+          <t>Not in scope of this MVP 1.1 release — enhancement later with a dedicated team. Traceability is already covered: every amendment writes the full old → new record with user and timestamp in the Application History (BRD section 3 action 6, SC6). A reason-code convention is a platform-wide edit-framework topic, to be taken up with the dedicated team if prioritised.</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -1047,12 +1098,12 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Not incorporated — new scope</t>
+          <t>To be discussed</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>STP behaviour: already in BRD v1.0 (flow + sections 3, 6). Decision matrix / delegated authority: proposed as a separate scope discussion.</t>
+          <t>Not in scope of this MVP 1.1 release — enhancement later with a dedicated team. The STP leg is already delivered in V1.1 (matched employer → automatic re-classification, recalculation, Rule Engine re-run and routing — sections 3 and flow). The formal STP decision matrix and delegated-authority routing are a dedicated design exercise for the follow-up scope.</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -1076,12 +1127,12 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Not incorporated — new scope</t>
+          <t>To be discussed</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Visibility of all recalculated values: already covered — BRD v1.0 sections 3-4, SC5/SC6. Delta-detection control: with item 4 in the new scope.</t>
+          <t>Not in scope of this MVP 1.1 release — enhancement later with a dedicated team. Visibility of every movement (ALOC, category, Rule Engine Result, Approve Limit Result, history before/after) is already in V1.1 (sections 3–4, SC5/SC6). Automated delta-detection and escalation join the item 4 initiative in the follow-up scope.</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -1100,22 +1151,22 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Repeat amendments are already bounded and visible by design. Every amendment re-runs the Rule Engine under the platform's shared re-run counter — an application that fails the Rule Engine more than twice is automatically rejected — and every amendment writes its own fully detailed step in the Application History (BRD section 3, SC6), so repeated activity is immediately visible to anyone reviewing the case. The action is restricted to authorised Credit users inside the controlled queue environment. A configurable repeat-amendment threshold with escalating authority is workable, but it belongs to the same authority-matrix design as item 4; we propose deciding it there so the rule is consistent across all queue edits.</t>
+          <t>In the approved V1.1 the Rule Engine re-runs with no cap, and there is no cap on repeat edits — the feature relies on controls rather than a hard limit: the edit sits inside the Bank's manual review layer, is restricted to authorised Credit users, and every amendment writes its own fully detailed step in the Application History (section 3, SC6), so repeated activity is immediately visible to anyone reviewing or approving the case. A configurable repeat-amendment control (threshold, escalation) is recommended as part of the follow-up control scope rather than this release.</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Not incorporated</t>
+          <t>To be discussed</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Bounding and traceability already covered — BRD v1.0 section 3 (re-run counter, per-edit audit), SC6. Configurable threshold: with the item 4 scope discussion.</t>
+          <t>Not in scope of this MVP 1.1 release — enhancement later with a dedicated team. V1.1 final: no cap on re-run (section 3 action 4); per-edit traceability covered (action 6, SC6). Configurable repeat-amendment threshold: follow-up control scope together with items 4 and 5.</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>BRD section 3 (re-run counter) — per-edit history steps (screen SC6)</t>
+          <t>BRD V1.1 section 3 — action 4 (no cap on re-run) and action 6 (per-edit history steps, SC6)</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr"/>
@@ -1129,7 +1180,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Confirmed — this is the existing behaviour. The counter counts business Rule Engine outcomes of the application; technical and integration failures are handled by the platform's error-handling and retry mechanisms and do not consume the counter or reject the customer. This is Day-1 platform behaviour that this feature re-uses unchanged; we will state it explicitly in the BRD for clarity.</t>
+          <t>Confirmed as platform behaviour: a customer is never rejected because of a system timeout, API failure or technical retry — technical and integration failures are handled by the platform's Day-1 error-handling and retry mechanisms, which apply uniformly to every function. In the approved V1.1 the Rule Engine re-run carries no cap (section 3 action 4), so no business re-run counter applies to this feature; the concern raised is fully addressed by design.</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -1139,12 +1190,12 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Existing platform behaviour — BRD v1.0 section 3 action 4; one clarification sentence added in v1.1.</t>
+          <t>Platform Day-1 behaviour. BRD V1.1 section 3 action 4: Rule Engine re-run with no cap — no counter consumed by this feature; technical failures handled by platform error handling.</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>BRD section 3, system actions table (action 4 — Rule Engine re-run and counter)</t>
+          <t>BRD V1.1 section 3, system actions table — action 4 (Rule Engine re-run, no cap)</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr"/>
@@ -1192,12 +1243,12 @@
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>Not incorporated — separate stream</t>
+          <t>To be discussed</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Monitoring source data: already covered — BRD v1.0 audit trail (section 3, SC6). Monitoring views: Bank reporting/control stream, with item 18.</t>
+          <t>Not in scope of this MVP 1.1 release — enhancement later with a dedicated team. All source data points (amendment counts, user, old/new classification, repeat patterns) are captured from day one in the audit trail and Application History (section 3, SC6). Monitoring views: Bank reporting/control stream, consolidated with item 18.</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -1221,12 +1272,12 @@
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Not incorporated — separate CR</t>
+          <t>To be discussed</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Out of this feature. Referenced in the BRD dependencies; matching quality of item 1 improves automatically with this stream.</t>
+          <t>Not in scope of this MVP 1.1 release — enhancement later with a dedicated team. The Empaneled Company List is a Bank-owned master with its own maintenance process; its governance, data dictionary and maker-checker apply to every consuming function — recommended as a dedicated change request. This feature consumes the master as-is and benefits automatically.</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -1366,12 +1417,12 @@
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>Not incorporated — platform NFR</t>
+          <t>To be discussed</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Governed by the Day-1 platform architecture; this feature adds no new integration pattern. No change to the BRD.</t>
+          <t>Not in scope of this MVP 1.1 release — enhancement later with a dedicated team. Non-functional, platform-level requirements governed by the Day-1 architecture; this feature introduces no new integration pattern. To be addressed as a platform resiliency topic with the dedicated team, not per feature.</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -1453,12 +1504,12 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Not incorporated — separate stream</t>
+          <t>To be discussed</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Source data covered (BRD v1.0 audit trail). Report delivery: Bank reporting stream together with item 9.</t>
+          <t>Not in scope of this MVP 1.1 release — enhancement later with a dedicated team. The reporting source data is produced from day one (audit trail / Application History). MIS delivery: Bank reporting stream, consolidated with item 9.</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -1487,12 +1538,12 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>BRD v1.1: both paragraphs included as governing statements (feature overview + section 3). Exception-routing conditions: with the item 4 initiative.</t>
+          <t>Incorporated in BRD V1.1 as enforced design rules rather than quoted text: the Employer matching rules table (section 2) states that classification is never taken from the typed text itself and that no confident match leaves the application N-ALOC (validation-first, exception-based), and section 3 action 7 states the one controlled transaction with no partial update. Exception-routing conditions: with the item 4 initiative.</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>BRD v1.1 — governing statements added to overview and section 3</t>
+          <t>BRD V1.1 — Employer matching rules table (section 2) + section 3 action 7 (controlled transaction)</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr"/>

</xml_diff>